<commit_message>
Update input data loading to treat CEPs, SKUs, and Sellers as strings
</commit_message>
<xml_diff>
--- a/input_ceps_skus.xlsx
+++ b/input_ceps_skus.xlsx
@@ -5,17 +5,17 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SKUs" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="CEPs" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="SELLERs" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1"/>
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -24,17 +24,18 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
-    <t xml:space="preserve">pelegrin</t>
+    <t xml:space="preserve">01409001</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -56,6 +57,13 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -74,7 +82,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
+  <cellStyleXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -98,24 +106,37 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="Normal 2" xfId="20"/>
   </cellStyles>
 </styleSheet>
 </file>
@@ -125,17 +146,387 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:A76"/>
+  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="n">
-        <v>2071060</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
-        <v>100358954</v>
+        <v>1922080</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1412239</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>1412260</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>1257670</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>1922080</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>1412260</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>1412239</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>2011202</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
+        <v>1870299</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
+        <v>1106541</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="n">
+        <v>1434279</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="n">
+        <v>500562</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="n">
+        <v>2084176</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="n">
+        <v>1440201</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="n">
+        <v>1106541</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="n">
+        <v>2089263</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="n">
+        <v>2085333</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="n">
+        <v>2046044</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="n">
+        <v>1106534</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="n">
+        <v>2084183</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="n">
+        <v>2089959</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="n">
+        <v>1922066</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="n">
+        <v>1770940</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="n">
+        <v>1440201</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="n">
+        <v>1458947</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="n">
+        <v>1458909</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="n">
+        <v>1873870</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="n">
+        <v>2003559</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="n">
+        <v>160674</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="n">
+        <v>1482157</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="n">
+        <v>2000718</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="n">
+        <v>1618457</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="n">
+        <v>1793307</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="n">
+        <v>1505528</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="n">
+        <v>1257670</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="n">
+        <v>1933796</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="0" t="n">
+        <v>1871081</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="0" t="n">
+        <v>1241082</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="0" t="n">
+        <v>1793505</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="0" t="n">
+        <v>1988741</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="n">
+        <v>1406238</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="n">
+        <v>1466683</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="0" t="n">
+        <v>937559</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0" t="n">
+        <v>2103723</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="0" t="n">
+        <v>1728651</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="0" t="n">
+        <v>2010427</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="0" t="n">
+        <v>1993622</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="0" t="n">
+        <v>1653496</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0" t="n">
+        <v>525411</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="0" t="n">
+        <v>1922066</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="0" t="n">
+        <v>1701654</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="0" t="n">
+        <v>2113715</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="0" t="n">
+        <v>1701654</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="0" t="n">
+        <v>1719321</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="0" t="n">
+        <v>1880588</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="0" t="n">
+        <v>1761863</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="0" t="n">
+        <v>1761726</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="0" t="n">
+        <v>1076851</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="0" t="n">
+        <v>89203</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="0" t="n">
+        <v>2053400</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="0" t="n">
+        <v>2069197</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="0" t="n">
+        <v>190640</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="0" t="n">
+        <v>652933</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="0" t="n">
+        <v>2116884</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="0" t="n">
+        <v>1922066</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="0" t="n">
+        <v>1531572</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="0" t="n">
+        <v>1907308</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="0" t="n">
+        <v>1964462</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="0" t="n">
+        <v>1759389</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="0" t="n">
+        <v>2106083</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="0" t="n">
+        <v>966061</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0" t="n">
+        <v>1789355</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="0" t="n">
+        <v>1938906</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="0" t="n">
+        <v>1106480</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="0" t="n">
+        <v>1874372</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="0" t="n">
+        <v>1950823</v>
       </c>
     </row>
   </sheetData>
@@ -154,17 +545,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="11.71"/>
+  </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="n">
-        <v>88134360</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
-        <v>22450200</v>
+    <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -184,17 +573,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
+    <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>